<commit_message>
Add new spreadsheet of my portfolio with a column to capture the RavenPack Entity ID
</commit_message>
<xml_diff>
--- a/how_to_guides/claude-cowork/portfolio_daily_impact_analysis/my_portfolio_YYYY_MM_DD-HH_MM.xlsx
+++ b/how_to_guides/claude-cowork/portfolio_daily_impact_analysis/my_portfolio_YYYY_MM_DD-HH_MM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\osanchez\Documents\MyDocuments\ClaudeCoWork\PortfolioDailyNews\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA86ECF5-10A3-4FF8-B573-EF2A29F73846}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05898018-76B8-47D3-8624-041C38C5D0E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="my_portfolio_template" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Ticker</t>
   </si>
@@ -110,6 +110,9 @@
   </si>
   <si>
     <t>Microsoft Corporation</t>
+  </si>
+  <si>
+    <t>RavenPack Entity ID</t>
   </si>
 </sst>
 </file>
@@ -479,7 +482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -487,13 +490,14 @@
     <col min="3" max="3" width="13.42578125" hidden="1" customWidth="1"/>
     <col min="4" max="5" width="13" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="8.5703125" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="34.42578125" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" customWidth="1"/>
-    <col min="9" max="9" width="13.28515625" customWidth="1"/>
-    <col min="10" max="10" width="17.85546875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" customWidth="1"/>
+    <col min="8" max="8" width="34.42578125" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" customWidth="1"/>
+    <col min="11" max="11" width="17.85546875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -513,19 +517,22 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -533,7 +540,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -541,7 +548,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -549,7 +556,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -557,7 +564,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -565,7 +572,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -573,7 +580,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -581,7 +588,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -589,7 +596,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -597,7 +604,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
Remove hiden columns from the spreadsheet my_portfolio
</commit_message>
<xml_diff>
--- a/how_to_guides/claude-cowork/portfolio_daily_impact_analysis/my_portfolio_YYYY_MM_DD-HH_MM.xlsx
+++ b/how_to_guides/claude-cowork/portfolio_daily_impact_analysis/my_portfolio_YYYY_MM_DD-HH_MM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\osanchez\Documents\MyDocuments\ClaudeCoWork\PortfolioDailyNews\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05898018-76B8-47D3-8624-041C38C5D0E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{089A53B5-801E-43A2-B0D8-2A020C7F97F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="my_portfolio_template" sheetId="1" r:id="rId1"/>
@@ -20,24 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Ticker</t>
   </si>
   <si>
     <t>Company Name</t>
-  </si>
-  <si>
-    <t>Market Cap</t>
-  </si>
-  <si>
-    <t>P/E</t>
-  </si>
-  <si>
-    <t>EPS</t>
-  </si>
-  <si>
-    <t>Yield</t>
   </si>
   <si>
     <t>Topics that could impact this company</t>
@@ -482,22 +470,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="36.42578125" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" hidden="1" customWidth="1"/>
-    <col min="4" max="5" width="13" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" customWidth="1"/>
-    <col min="8" max="8" width="34.42578125" customWidth="1"/>
-    <col min="9" max="9" width="11.7109375" customWidth="1"/>
-    <col min="10" max="10" width="13.28515625" customWidth="1"/>
-    <col min="11" max="11" width="17.85546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="37" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="34.42578125" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -505,111 +490,99 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="B3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>14</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>16</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>18</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>20</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>22</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B10" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>24</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B11" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>